<commit_message>
formulario dos | admin inter formulario
</commit_message>
<xml_diff>
--- a/requerimientos/adjuntos/ADMIN-APLICATIVO_WEB/Plantilla de información de persona_2026_06_16_13_27_44.xlsx
+++ b/requerimientos/adjuntos/ADMIN-APLICATIVO_WEB/Plantilla de información de persona_2026_06_16_13_27_44.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/melquiromero/Documents/GitHub/SCA-CIDE/requerimientos/adjuntos/ADMIN-APLICATIVO_WEB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3692D3E3-8093-CC46-A17E-071FD7AB3180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B31CACD-66C0-4F4F-BA15-F6136C068C52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-44800" yWindow="2880" windowWidth="44800" windowHeight="24600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plantilla de información de ..." sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4151" uniqueCount="1188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4177" uniqueCount="1196">
   <si>
     <t>Regla</t>
   </si>
@@ -3600,6 +3600,30 @@
   </si>
   <si>
     <t>SENA CIUDAD VERDE/ADMINISTRATIVOS/TICs</t>
+  </si>
+  <si>
+    <t>KAREN TATIANA PARRAGA TORO</t>
+  </si>
+  <si>
+    <t>Jazmin Aurora Vega Perez</t>
+  </si>
+  <si>
+    <t>Cristian Felipe Aguilar Reyes</t>
+  </si>
+  <si>
+    <t>kparraga@sena.edu.co</t>
+  </si>
+  <si>
+    <t>312 5743035</t>
+  </si>
+  <si>
+    <t>jvegap@sena.edu.co</t>
+  </si>
+  <si>
+    <t>321 3720336</t>
+  </si>
+  <si>
+    <t>cfaguilar@sena.edu.co</t>
   </si>
 </sst>
 </file>
@@ -3979,7 +4003,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K503"/>
+  <dimension ref="A1:K506"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" customWidth="1"/>
@@ -21386,6 +21410,111 @@
         <v>5585</v>
       </c>
     </row>
+    <row r="504" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A504">
+        <v>1073669651</v>
+      </c>
+      <c r="B504" t="s">
+        <v>1188</v>
+      </c>
+      <c r="C504" t="s">
+        <v>21</v>
+      </c>
+      <c r="D504" t="s">
+        <v>1022</v>
+      </c>
+      <c r="E504" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F504" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G504" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H504" t="s">
+        <v>19</v>
+      </c>
+      <c r="I504" t="s">
+        <v>1191</v>
+      </c>
+      <c r="J504" t="s">
+        <v>1192</v>
+      </c>
+      <c r="K504">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="505" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A505">
+        <v>1000185797</v>
+      </c>
+      <c r="B505" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C505" t="s">
+        <v>21</v>
+      </c>
+      <c r="D505" t="s">
+        <v>1022</v>
+      </c>
+      <c r="E505" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F505" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G505" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H505" t="s">
+        <v>19</v>
+      </c>
+      <c r="I505" t="s">
+        <v>1193</v>
+      </c>
+      <c r="J505" t="s">
+        <v>1194</v>
+      </c>
+      <c r="K505">
+        <v>2213</v>
+      </c>
+    </row>
+    <row r="506" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A506">
+        <v>1011086205</v>
+      </c>
+      <c r="B506" t="s">
+        <v>1190</v>
+      </c>
+      <c r="C506" t="s">
+        <v>21</v>
+      </c>
+      <c r="D506" t="s">
+        <v>1022</v>
+      </c>
+      <c r="E506" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F506" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G506" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H506" t="s">
+        <v>19</v>
+      </c>
+      <c r="I506" t="s">
+        <v>1195</v>
+      </c>
+      <c r="J506">
+        <v>3114625263</v>
+      </c>
+      <c r="K506">
+        <v>2218</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A1:A1048576">

</xml_diff>